<commit_message>
docs: restore prior guidance values in EA evaluation workbook
</commit_message>
<xml_diff>
--- a/tools/ea-evaluation/GSM_EA_综合评估工具表_v1.0.xlsx
+++ b/tools/ea-evaluation/GSM_EA_综合评估工具表_v1.0.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="综合评估" sheetId="1" r:id="Ra350960396bc473e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分政策" sheetId="2" r:id="Ra6d8e879e2ca4ccc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略与验证" sheetId="3" r:id="R8714f88551d9479a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="综合评估" sheetId="1" r:id="R987fae81d1494bfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="评分政策" sheetId="2" r:id="Rf4d5bdca6bf04a33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="策略与验证" sheetId="3" r:id="Rbaff43140254486e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -26,7 +26,7 @@
     <x:numFmt numFmtId="207" formatCode="0.0%"/>
     <x:numFmt numFmtId="208" formatCode="0.00%"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -64,8 +64,14 @@
       <x:color rgb="FF243746"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="6">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -87,6 +93,11 @@
         <x:fgColor rgb="FFEDF3F8"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF233D58"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="2">
     <x:border/>
@@ -99,7 +110,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="39">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -201,6 +212,10 @@
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -211,7 +226,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -221,7 +236,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -231,7 +246,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -241,7 +256,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE8E7"/>
         </x:patternFill>
       </x:fill>
@@ -254,14 +269,14 @@
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CF"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
     <x:dxf>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF0CF"/>
         </x:patternFill>
       </x:fill>
@@ -2332,7 +2347,7 @@
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="2"/>
       <x:c r="B3" s="4" t="str">
-        <x:v>事前冻结；每批另存</x:v>
+        <x:v>已给建议见下方参考表</x:v>
       </x:c>
       <x:c r="C3" s="4"/>
       <x:c r="D3" s="4"/>
@@ -2654,7 +2669,7 @@
     <x:row r="25" ht="27" customHeight="1">
       <x:c r="A25" s="2"/>
       <x:c r="B25" s="9" t="str">
-        <x:v>正式评分锚点（初始留空）</x:v>
+        <x:v>本批正式评分锚点</x:v>
       </x:c>
       <x:c r="C25" s="9"/>
       <x:c r="D25" s="10"/>
@@ -2676,7 +2691,7 @@
       <x:c r="G26" s="5"/>
       <x:c r="H26" s="2"/>
       <x:c r="I26" s="6" t="str">
-        <x:v>满分净利润 USD；&gt;0</x:v>
+        <x:v>已有建议：净利需为正，结合本金与测试时长；满分金额 P_target 仍需本批登记。</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
@@ -2691,7 +2706,7 @@
       <x:c r="G27" s="5"/>
       <x:c r="H27" s="2"/>
       <x:c r="I27" s="6" t="str">
-        <x:v>满分回撤百分数；输入 5 表示 5%</x:v>
+        <x:v>旧版已有目标：最大相对净值DD≤15%；这不是自动满分，D_good须说明依据。</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
@@ -2706,7 +2721,7 @@
       <x:c r="G28" s="5"/>
       <x:c r="H28" s="2"/>
       <x:c r="I28" s="6" t="str">
-        <x:v>零分回撤百分数；必须 &gt;D_good</x:v>
+        <x:v>旧版已有边界：15%～30%严格复核，&gt;30%拒绝；D_bad仍需登记。</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
@@ -2721,7 +2736,7 @@
       <x:c r="G29" s="5"/>
       <x:c r="H29" s="2"/>
       <x:c r="I29" s="6" t="str">
-        <x:v>满分原生 PF；&gt;1</x:v>
+        <x:v>已有建议：PF 1.3～1.8作诊断参考，不设1.8上限；F_target是另一项满分目标。</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
@@ -2736,7 +2751,7 @@
       <x:c r="G30" s="5"/>
       <x:c r="H30" s="2"/>
       <x:c r="I30" s="6" t="str">
-        <x:v>正整数，旧版主区间至少 101</x:v>
+        <x:v>已有建议：200～500笔；旧版主区间至少101笔。N_target须登记，达到后封顶。</x:v>
       </x:c>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
@@ -2751,7 +2766,7 @@
       <x:c r="G31" s="5"/>
       <x:c r="H31" s="2"/>
       <x:c r="I31" s="6" t="str">
-        <x:v>满分成本 USD / 往返标准手；≥0</x:v>
+        <x:v>已有建议：成本后净期望 / 同口径每完整交易成本，目标参考3～5倍。</x:v>
       </x:c>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
@@ -2766,7 +2781,7 @@
       <x:c r="G32" s="5"/>
       <x:c r="H32" s="2"/>
       <x:c r="I32" s="6" t="str">
-        <x:v>零分成本；必须 &gt;C_good</x:v>
+        <x:v>C_good/C_bad单位为USD/往返标准手；不能把3～5倍净期望成本比直接填进来。</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
@@ -3096,7 +3111,7 @@
       <x:c r="G55" s="5"/>
       <x:c r="H55" s="2"/>
       <x:c r="I55" s="6" t="str">
-        <x:v>综合分只用于同条件诊断。80%表示80/100，不是胜率或自动通过线。</x:v>
+        <x:v>建议值已收录于69行起；正式评分目标与建议范围分开，80%不等于胜率。</x:v>
       </x:c>
     </x:row>
     <x:row r="56" ht="23" customHeight="1">
@@ -3252,6 +3267,302 @@
       <x:c r="H66" s="2"/>
       <x:c r="I66" s="6" t="str">
         <x:v>https://github.com/chanteck123-ux/gsm-mt5-indicators</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="27" customHeight="1">
+      <x:c r="B69" s="36" t="str">
+        <x:v>你之前提供的建议值</x:v>
+      </x:c>
+      <x:c r="C69" s="36"/>
+      <x:c r="D69" s="36"/>
+      <x:c r="E69" s="36"/>
+      <x:c r="F69" s="36"/>
+      <x:c r="G69" s="36"/>
+    </x:row>
+    <x:row r="70" ht="26" customHeight="1">
+      <x:c r="B70" s="37" t="str">
+        <x:v>评估项目</x:v>
+      </x:c>
+      <x:c r="C70" s="37" t="str">
+        <x:v>已有建议 / 已保存目标</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="26" customHeight="1">
+      <x:c r="B71" s="2" t="str">
+        <x:v>净利润 USD</x:v>
+      </x:c>
+      <x:c r="C71" s="2" t="str">
+        <x:v>须为正</x:v>
+      </x:c>
+      <x:c r="D71" s="2"/>
+      <x:c r="E71" s="2"/>
+      <x:c r="F71" s="2"/>
+      <x:c r="G71" s="2"/>
+      <x:c r="H71" s="2"/>
+      <x:c r="I71" s="6" t="str">
+        <x:v>旧版基本条件；同时比较本金、时长、风险和提款后持续运作。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="26" customHeight="1">
+      <x:c r="B72" s="2" t="str">
+        <x:v>最大相对净值回撤</x:v>
+      </x:c>
+      <x:c r="C72" s="2" t="str">
+        <x:v>目标≤15%</x:v>
+      </x:c>
+      <x:c r="D72" s="2"/>
+      <x:c r="E72" s="2"/>
+      <x:c r="F72" s="2"/>
+      <x:c r="G72" s="2"/>
+      <x:c r="H72" s="2"/>
+      <x:c r="I72" s="6" t="str">
+        <x:v>旧版已选项目目标；不是未来损失上限，也不是评分满分值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="26" customHeight="1">
+      <x:c r="B73" s="2" t="str">
+        <x:v>回撤复核与拒绝边界</x:v>
+      </x:c>
+      <x:c r="C73" s="2" t="str">
+        <x:v>15%～30%复核；&gt;30%拒绝</x:v>
+      </x:c>
+      <x:c r="D73" s="2"/>
+      <x:c r="E73" s="2"/>
+      <x:c r="F73" s="2"/>
+      <x:c r="G73" s="2"/>
+      <x:c r="H73" s="2"/>
+      <x:c r="I73" s="6" t="str">
+        <x:v>仅适用旧版当前主区间政策；不自动套用V1.2。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="26" customHeight="1">
+      <x:c r="B74" s="2" t="str">
+        <x:v>原生 Profit Factor</x:v>
+      </x:c>
+      <x:c r="C74" s="2" t="str">
+        <x:v>1.3～1.8</x:v>
+      </x:c>
+      <x:c r="D74" s="2"/>
+      <x:c r="E74" s="2"/>
+      <x:c r="F74" s="2"/>
+      <x:c r="G74" s="2"/>
+      <x:c r="H74" s="2"/>
+      <x:c r="I74" s="6" t="str">
+        <x:v>诊断参考；不设1.8上限，PF高也须核对成本、样本与多次选择。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75" ht="26" customHeight="1">
+      <x:c r="B75" s="2" t="str">
+        <x:v>完整交易数</x:v>
+      </x:c>
+      <x:c r="C75" s="2" t="str">
+        <x:v>建议200～500笔</x:v>
+      </x:c>
+      <x:c r="D75" s="2"/>
+      <x:c r="E75" s="2"/>
+      <x:c r="F75" s="2"/>
+      <x:c r="G75" s="2"/>
+      <x:c r="H75" s="2"/>
+      <x:c r="I75" s="6" t="str">
+        <x:v>旧版主区间&gt;100，至少101；建议范围不是上限，也不证明样本独立。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76" ht="26" customHeight="1">
+      <x:c r="B76" s="2" t="str">
+        <x:v>原生 Recovery</x:v>
+      </x:c>
+      <x:c r="C76" s="2" t="str">
+        <x:v>&gt;3.0</x:v>
+      </x:c>
+      <x:c r="D76" s="2"/>
+      <x:c r="E76" s="2"/>
+      <x:c r="F76" s="2"/>
+      <x:c r="G76" s="2"/>
+      <x:c r="H76" s="2"/>
+      <x:c r="I76" s="6" t="str">
+        <x:v>旧版已选硬条件；使用最大余额DD，另看Equity Recovery。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77" ht="26" customHeight="1">
+      <x:c r="B77" s="2" t="str">
+        <x:v>成本后净期望 / 成本</x:v>
+      </x:c>
+      <x:c r="C77" s="2" t="str">
+        <x:v>参考3～5倍</x:v>
+      </x:c>
+      <x:c r="D77" s="2"/>
+      <x:c r="E77" s="2"/>
+      <x:c r="F77" s="2"/>
+      <x:c r="G77" s="2"/>
+      <x:c r="H77" s="2"/>
+      <x:c r="I77" s="6" t="str">
+        <x:v>统一为每完整交易USD口径；成本为0或未知时未定义。不是USD/往返手锚点。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78" ht="26" customHeight="1">
+      <x:c r="B78" s="2" t="str">
+        <x:v>评分权重</x:v>
+      </x:c>
+      <x:c r="C78" s="2" t="str">
+        <x:v>35 / 25 / 20 / 10 / 10</x:v>
+      </x:c>
+      <x:c r="D78" s="2"/>
+      <x:c r="E78" s="2"/>
+      <x:c r="F78" s="2"/>
+      <x:c r="G78" s="2"/>
+      <x:c r="H78" s="2"/>
+      <x:c r="I78" s="6" t="str">
+        <x:v>对应净利润、净值DD、PF、完整交易数、每往返手成本，单位%。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79" ht="26" customHeight="1">
+      <x:c r="B79" s="2" t="str">
+        <x:v>持续运作与强平</x:v>
+      </x:c>
+      <x:c r="C79" s="2" t="str">
+        <x:v>核对Stop Out及异常停机</x:v>
+      </x:c>
+      <x:c r="D79" s="2"/>
+      <x:c r="E79" s="2"/>
+      <x:c r="F79" s="2"/>
+      <x:c r="G79" s="2"/>
+      <x:c r="H79" s="2"/>
+      <x:c r="I79" s="6" t="str">
+        <x:v>新闻或风险规则正常暂停需核对恢复，不为凑笔数强行开单。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="80" ht="26" customHeight="1">
+      <x:c r="B80" s="2" t="str">
+        <x:v>V1.2 初始研究资金</x:v>
+      </x:c>
+      <x:c r="C80" s="2" t="str">
+        <x:v>500 USD</x:v>
+      </x:c>
+      <x:c r="D80" s="2"/>
+      <x:c r="E80" s="2"/>
+      <x:c r="F80" s="2"/>
+      <x:c r="G80" s="2"/>
+      <x:c r="H80" s="2"/>
+      <x:c r="I80" s="6" t="str">
+        <x:v>来自V1.2独立计划；不是本表对所有项目的默认资金。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81" ht="26" customHeight="1">
+      <x:c r="B81" s="2" t="str">
+        <x:v>V1.2 连续研究区间</x:v>
+      </x:c>
+      <x:c r="C81" s="2" t="str">
+        <x:v>12个完整自然月</x:v>
+      </x:c>
+      <x:c r="D81" s="2"/>
+      <x:c r="E81" s="2"/>
+      <x:c r="F81" s="2"/>
+      <x:c r="G81" s="2"/>
+      <x:c r="H81" s="2"/>
+      <x:c r="I81" s="6" t="str">
+        <x:v>事前固定连续区间，无追加资金、无重置；亏损及无交易月份均计入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="82" ht="26" customHeight="1">
+      <x:c r="B82" s="2" t="str">
+        <x:v>V1.2 成本后净利润目标</x:v>
+      </x:c>
+      <x:c r="C82" s="2" t="str">
+        <x:v>合计≥12,000 USD</x:v>
+      </x:c>
+      <x:c r="D82" s="2"/>
+      <x:c r="E82" s="2"/>
+      <x:c r="F82" s="2"/>
+      <x:c r="G82" s="2"/>
+      <x:c r="H82" s="2"/>
+      <x:c r="I82" s="6" t="str">
+        <x:v>挑战目标，尚未被证明达成；不能替换其他项目评分满分值。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83" ht="26" customHeight="1">
+      <x:c r="B83" s="2" t="str">
+        <x:v>V1.2 月均净利润目标</x:v>
+      </x:c>
+      <x:c r="C83" s="2" t="str">
+        <x:v>月均≥1,000 USD</x:v>
+      </x:c>
+      <x:c r="D83" s="2"/>
+      <x:c r="E83" s="2"/>
+      <x:c r="F83" s="2"/>
+      <x:c r="G83" s="2"/>
+      <x:c r="H83" s="2"/>
+      <x:c r="I83" s="6" t="str">
+        <x:v>不是每月固定盈利承诺；连续账户与月末提款账户分别完整测试。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="84" ht="26" customHeight="1">
+      <x:c r="B84" s="2"/>
+      <x:c r="C84" s="2"/>
+      <x:c r="D84" s="2"/>
+      <x:c r="E84" s="2"/>
+      <x:c r="F84" s="2"/>
+      <x:c r="G84" s="2"/>
+      <x:c r="H84" s="2"/>
+      <x:c r="I84" s="6"/>
+    </x:row>
+    <x:row r="85" ht="26" customHeight="1">
+      <x:c r="B85" s="2" t="str">
+        <x:v>§13.10 完整评分算例</x:v>
+      </x:c>
+      <x:c r="C85" s="2" t="str">
+        <x:v>保留为演算示例</x:v>
+      </x:c>
+      <x:c r="D85" s="2"/>
+      <x:c r="E85" s="2"/>
+      <x:c r="F85" s="2"/>
+      <x:c r="G85" s="2"/>
+      <x:c r="H85" s="2"/>
+      <x:c r="I85" s="6" t="str">
+        <x:v>P=1000 USD；D_good=5%、D_bad=30%；F=2；N=200；C_good=10、C_bad=30 USD/RT。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="86" ht="26" customHeight="1">
+      <x:c r="B86" s="2" t="str">
+        <x:v>算例的使用身份</x:v>
+      </x:c>
+      <x:c r="C86" s="2" t="str">
+        <x:v>未自动选作本批正式值</x:v>
+      </x:c>
+      <x:c r="D86" s="2"/>
+      <x:c r="E86" s="2"/>
+      <x:c r="F86" s="2"/>
+      <x:c r="G86" s="2"/>
+      <x:c r="H86" s="2"/>
+      <x:c r="I86" s="6" t="str">
+        <x:v>建议与既有目标并非没有提供；正式锚点须按适用项目和本批条件登记。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88" ht="26" customHeight="1">
+      <x:c r="B88" s="38" t="str">
+        <x:v>建议值来源</x:v>
+      </x:c>
+      <x:c r="C88" s="38"/>
+      <x:c r="D88" s="38"/>
+      <x:c r="E88" s="38"/>
+      <x:c r="F88" s="38"/>
+      <x:c r="G88" s="38"/>
+      <x:c r="H88" s="38"/>
+      <x:c r="I88" s="38" t="str">
+        <x:v>本次对话既有用户资料；旧版计划§11.1、§11.3、§11.4、§13.10。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="89" ht="26" customHeight="1">
+      <x:c r="B89" s="38" t="str">
+        <x:v>V1.2 目标来源</x:v>
+      </x:c>
+      <x:c r="C89" s="38"/>
+      <x:c r="D89" s="38"/>
+      <x:c r="E89" s="38"/>
+      <x:c r="F89" s="38"/>
+      <x:c r="G89" s="38"/>
+      <x:c r="H89" s="38"/>
+      <x:c r="I89" s="38" t="str">
+        <x:v>https://github.com/chanteck123-ux/TX-AI---EA-GOLD-Trading/blob/8f0250bc0f867ebebfe08aab872587ca5e42d5da/开发交易头脑EA/交易头脑v1.2/docs/PLAN_CN.md</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>